<commit_message>
Update data and analysis
</commit_message>
<xml_diff>
--- a/Clean_Grievance_Sample.xlsx
+++ b/Clean_Grievance_Sample.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="46">
   <si>
     <t>PROVINCE</t>
   </si>
@@ -794,7 +794,7 @@
       <c r="E15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -997,8 +997,14 @@
       <c r="E25" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>11</v>
+      <c r="F25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">

</xml_diff>